<commit_message>
docs(voice): Alpha and Prawn Again exempt from the 'we' rule; You check tab updated (160 lines left to rewrite)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KktbqAKqtW6yYf3NiibPQe
</commit_message>
<xml_diff>
--- a/storm-directive/Card_Copy_Draft_All.xlsx
+++ b/storm-directive/Card_Copy_Draft_All.xlsx
@@ -11617,14 +11617,14 @@
           <t>Pop quiz: who is high-value? Not them. They fail. You pass.</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11652,14 +11652,14 @@
           <t>Everyone sees your energy now. Mogging the whole room, live.</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11687,14 +11687,14 @@
           <t>Never look back. Unless your past is on fire. Then look. Admire.</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11722,14 +11722,14 @@
           <t>Let them run. Every one of them is advertising you. Free reach.</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11757,14 +11757,14 @@
           <t>CEO energy. Let them knock each other out while you look busy.</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11792,14 +11792,14 @@
           <t>Leave a legacy. Seventy per cent of greatness happens after you go.</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11827,14 +11827,14 @@
           <t>Grow the network. Everyone at the end of the chain works for you.</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11862,14 +11862,14 @@
           <t>Decoys. Plenty more eggs in the sea. Not that you need them.</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11897,14 +11897,14 @@
           <t>Big guy charging? Stay locked in. A stuck man cannot out-frame you.</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11932,14 +11932,14 @@
           <t>Everyone freezes under pressure. Except you. That is sigma behaviour.</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -11967,14 +11967,14 @@
           <t>Every top guy needs a wingman. This one never outshines you. Ideal.</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12002,14 +12002,14 @@
           <t>Timeout. Reset your frame. Breathe through the nose. Mewing. Go.</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12037,14 +12037,14 @@
           <t>That one disrespected you. Note the face. Ratio it into the ground.</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12072,14 +12072,14 @@
           <t>Real talk: blades are a personality. You have one now.</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12107,14 +12107,14 @@
           <t>Every star has an entourage. You are a ten. Act like it.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12142,14 +12142,14 @@
           <t>Patience is a weapon. Don't chase. Let them come to you.</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12177,14 +12177,14 @@
           <t>Go over the competition. They are not even in your league.</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12212,14 +12212,14 @@
           <t>Leave a legacy wherever you swim. Alphas mark territory.</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12247,14 +12247,14 @@
           <t>Everything revolves around you. Correct. The egg will work that out.</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12282,14 +12282,14 @@
           <t>Your strength is its strength. Mogging by proxy. Own it.</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12317,14 +12317,14 @@
           <t>Mass is frame. Bulking arc. You mog the competition by volume.</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12352,14 +12352,14 @@
           <t>Do not chase, attract. Everything comes to you now. Law of attraction.</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12387,14 +12387,14 @@
           <t>Length is a mindset, and you have it. Looksmaxxing, but for reach.</t>
         </is>
       </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12422,14 +12422,14 @@
           <t>Leave your mark. High-value men linger. Let that sink in.</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12457,14 +12457,14 @@
           <t>Clingy is low-value. Unless they cling to you. Then it is frame.</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12492,14 +12492,14 @@
           <t>Pull them in. Close the deal. Never chase. Make them come to you.</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12527,14 +12527,14 @@
           <t>Rule four: boundaries. Nobody crosses your lane. Not even a ten.</t>
         </is>
       </c>
-      <c r="F28" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12562,14 +12562,14 @@
           <t>Hit and step back. Never let them see you need them. Frame.</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12597,14 +12597,14 @@
           <t>Consolidate. Stop spreading yourself thin. Monogamy, for pellets.</t>
         </is>
       </c>
-      <c r="F30" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12632,14 +12632,14 @@
           <t>Rule seven: cover your six. A ten respects a man who looks back.</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12667,14 +12667,14 @@
           <t>Establish dominance. Push them out of your frame. Mog them.</t>
         </is>
       </c>
-      <c r="F32" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12702,14 +12702,14 @@
           <t>They crash into each other. Weak frame. Not your problem, king.</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12737,14 +12737,14 @@
           <t>Grip it like you mean it. Weak grip, weak life. Firm handshake.</t>
         </is>
       </c>
-      <c r="F34" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12772,14 +12772,14 @@
           <t>Use your network. Your enemy is your tool. Leverage, champ.</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12807,14 +12807,14 @@
           <t>Persistence. Three bites in, 80% quit. Not you. You are the 20%.</t>
         </is>
       </c>
-      <c r="F36" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12842,14 +12842,14 @@
           <t>Your impact spreads. That is influence, brother. Nine out of ten.</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12877,14 +12877,14 @@
           <t>Bank your nuts. Release on purpose. Semen retention, basically.</t>
         </is>
       </c>
-      <c r="F38" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12912,14 +12912,14 @@
           <t>They swarm you because you're elite. Snap, snap, snap. Abundance.</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12947,14 +12947,14 @@
           <t>Keep your enemies closer. Then use them as a shield. Sigma move.</t>
         </is>
       </c>
-      <c r="F40" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -12982,14 +12982,14 @@
           <t>Nobody touches you. You're a ten. Act like it. Eight, minimum.</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13017,14 +13017,14 @@
           <t>Your space is sacred. Small men crowd. Big men blast. Write that.</t>
         </is>
       </c>
-      <c r="F42" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13052,14 +13052,14 @@
           <t>Network through your best contact. 80% of success is who's near you.</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13087,14 +13087,14 @@
           <t>Leave an impression. She'll still see you after you've left. Aura.</t>
         </is>
       </c>
-      <c r="F44" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13122,14 +13122,14 @@
           <t>They crash, you profit. 64% of wealth is other men's errors.</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13157,14 +13157,14 @@
           <t>Ten closes and the room is yours. That's the funnel. Trust it.</t>
         </is>
       </c>
-      <c r="F46" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13192,14 +13192,14 @@
           <t>Reset your mindset. Winners reboot daily. 4am alarm energy.</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13227,14 +13227,14 @@
           <t>Every scrap of you is an asset. Leave nothing unmonetised.</t>
         </is>
       </c>
-      <c r="F48" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13262,14 +13262,14 @@
           <t>Never look back. Except to mog whatever's chasing you.</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13297,14 +13297,14 @@
           <t>Panic is for them. You're the calm one. Locked in. Always.</t>
         </is>
       </c>
-      <c r="F50" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13332,14 +13332,14 @@
           <t>Real talk: sometimes you do chase. Outbound only. Not with eggs.</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13367,14 +13367,14 @@
           <t>Your network is your net worth. Literally. Lines everywhere.</t>
         </is>
       </c>
-      <c r="F52" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13402,14 +13402,14 @@
           <t>Don't chase, attract. They come to you. Reel them in.</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13437,14 +13437,14 @@
           <t>Everywhere you go, you own. Expansion mindset. Mark the territory.</t>
         </is>
       </c>
-      <c r="F54" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13472,14 +13472,14 @@
           <t>Five touches and they're yours. Brand them. That's attraction.</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13507,14 +13507,14 @@
           <t>Drain them dry. Take what's yours. 100% retention. Provider energy.</t>
         </is>
       </c>
-      <c r="F56" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13542,14 +13542,14 @@
           <t>Eight targets. Zero hesitation. Shooting your shot, eight times.</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13577,14 +13577,14 @@
           <t>Don't chase. Attract. They come to you. Works on the egg. Works on these.</t>
         </is>
       </c>
-      <c r="F58" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13612,14 +13612,14 @@
           <t>Convert your rivals into employees. That's mogging, technically.</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13647,14 +13647,14 @@
           <t>Bring your exes back as decoys. 0% of them say no. I checked. Twice.</t>
         </is>
       </c>
-      <c r="F60" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13682,14 +13682,14 @@
           <t>Everyone wants to be on your team. 100% conversion. A ten notices that.</t>
         </is>
       </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13717,14 +13717,14 @@
           <t>Rule eleven: let your reputation precede you. Ideally on fire.</t>
         </is>
       </c>
-      <c r="F62" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13752,14 +13752,14 @@
           <t>Every flame in the room is yours now. That's ownership. That's sigma.</t>
         </is>
       </c>
-      <c r="F63" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13787,14 +13787,14 @@
           <t>Inner circle only. Keep your people close and the rest weak. Frame.</t>
         </is>
       </c>
-      <c r="F64" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13822,14 +13822,14 @@
           <t>Their losses, your assets. Provider energy. Let it compound.</t>
         </is>
       </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13857,14 +13857,14 @@
           <t>Three wins and you're untouchable. Bullets are just protein.</t>
         </is>
       </c>
-      <c r="F66" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13892,14 +13892,14 @@
           <t>Stretch them. Push past limits. Theirs, not yours. Looksmaxxing, sort of.</t>
         </is>
       </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13927,14 +13927,14 @@
           <t>Use the walls. Use everything. The walls work for you now. Locked in.</t>
         </is>
       </c>
-      <c r="F68" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13962,14 +13962,14 @@
           <t>Know your weight class. Then hit below it. Hard. That's alpha.</t>
         </is>
       </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -13997,14 +13997,14 @@
           <t>Build walls, not bridges. Protect your peace. And your jawline.</t>
         </is>
       </c>
-      <c r="F70" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14032,14 +14032,14 @@
           <t>Your wins should splash on everyone nearby. Spread the value.</t>
         </is>
       </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14067,14 +14067,14 @@
           <t>You are the ammunition. Aim at what you want. Then take it. Sigma.</t>
         </is>
       </c>
-      <c r="F72" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14102,14 +14102,14 @@
           <t>Sometimes you overdeliver. Statistically, I always overdeliver.</t>
         </is>
       </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14137,14 +14137,14 @@
           <t>Build your frame. Literally. Bullets are protein for alphas.</t>
         </is>
       </c>
-      <c r="F74" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14172,14 +14172,14 @@
           <t>Rebrand what you steal. That's not theft, it's a personal brand.</t>
         </is>
       </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14207,14 +14207,14 @@
           <t>Triple your reach. Bigger radius, bigger mog. Simple maths.</t>
         </is>
       </c>
-      <c r="F76" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14242,14 +14242,14 @@
           <t>Even the mines grind. If a mine can hustle, so can you.</t>
         </is>
       </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14277,14 +14277,14 @@
           <t>Let them carry your work home. Passive income. Mostly explosions.</t>
         </is>
       </c>
-      <c r="F78" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14312,14 +14312,14 @@
           <t>Rest days are for betas. If you must stop, stop armed.</t>
         </is>
       </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14347,14 +14347,14 @@
           <t>Long distance only works if you're high value. You are. Barely.</t>
         </is>
       </c>
-      <c r="F80" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14382,14 +14382,14 @@
           <t>Even your twin has a side hustle. Respect the grind.</t>
         </is>
       </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14417,14 +14417,14 @@
           <t>Scale the team. Delegate the sweeping. You're the CEO now.</t>
         </is>
       </c>
-      <c r="F82" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14452,14 +14452,14 @@
           <t>Leave them thinking about you. They always do. I assume.</t>
         </is>
       </c>
-      <c r="F83" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14487,14 +14487,14 @@
           <t>Surround yourself with yes-men. They amplify you. Yes. Exactly.</t>
         </is>
       </c>
-      <c r="F84" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14522,14 +14522,14 @@
           <t>Even your leftovers should work for you. Passive income, but balloons.</t>
         </is>
       </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14557,14 +14557,14 @@
           <t>Let them fight for the corner office. You stay above it. Sigma.</t>
         </is>
       </c>
-      <c r="F86" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14592,14 +14592,14 @@
           <t>Every breakup makes you stronger. 76% stronger, minimum. Science.</t>
         </is>
       </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14627,14 +14627,14 @@
           <t>Outsource your pain. Real leaders delegate suffering. I wrote the book.</t>
         </is>
       </c>
-      <c r="F88" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14662,14 +14662,14 @@
           <t>Everyone is connected. Six degrees from losing to you. Ratio.</t>
         </is>
       </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14697,14 +14697,14 @@
           <t>Loyalty is a liability. For them. Not for you. You are a free agent.</t>
         </is>
       </c>
-      <c r="F90" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14732,14 +14732,14 @@
           <t>Use your haters as a wall. Haters are a resource. Let that sink in.</t>
         </is>
       </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14767,14 +14767,14 @@
           <t>Capture their output. Own it. Now it is your content. Monetise.</t>
         </is>
       </c>
-      <c r="F92" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14802,14 +14802,14 @@
           <t>Protect the asset. You are the asset. Bubble-wrapped. High-value.</t>
         </is>
       </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14837,14 +14837,14 @@
           <t>Let them work for you. Free labour. Rolling free labour. Ten out of ten.</t>
         </is>
       </c>
-      <c r="F94" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14872,14 +14872,14 @@
           <t>Do not wait for the date. Make the date come to you. Attract, never chase.</t>
         </is>
       </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14907,14 +14907,14 @@
           <t>Stack your wins. Third win pays double. Fact. I read it somewhere.</t>
         </is>
       </c>
-      <c r="F96" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14942,14 +14942,14 @@
           <t>Pain is a delayed invoice. And you negotiated it down. Alpha move.</t>
         </is>
       </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -14977,14 +14977,14 @@
           <t>Wolves hunt in packs. You are a wolf. Basically. Alpha wolf.</t>
         </is>
       </c>
-      <c r="F98" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15012,14 +15012,14 @@
           <t>Rule one: leave a decoy. Let them simp for the wrong you. Boom.</t>
         </is>
       </c>
-      <c r="F99" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15047,14 +15047,14 @@
           <t>Seven on the decoy. Crowd rating: nine. Your frame did that.</t>
         </is>
       </c>
-      <c r="F100" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15082,14 +15082,14 @@
           <t>Toss them a toy. Chasing noise is beta behaviour. You? Locked in.</t>
         </is>
       </c>
-      <c r="F101" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15117,14 +15117,14 @@
           <t>Two of you. Double the value. A ten would swipe both. Probably.</t>
         </is>
       </c>
-      <c r="F102" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15152,14 +15152,14 @@
           <t>Fear is respect, fast-tracked. Real talk: they should be scared of you.</t>
         </is>
       </c>
-      <c r="F103" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15187,14 +15187,14 @@
           <t>Panic is viral. Let them do your marketing. You are the content.</t>
         </is>
       </c>
-      <c r="F104" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15222,14 +15222,14 @@
           <t>Sixty-four per cent of losers trip over other losers. Stay in your lane.</t>
         </is>
       </c>
-      <c r="F105" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15257,14 +15257,14 @@
           <t>Passive income. Bait that breeds bait. You sleep, it grinds.</t>
         </is>
       </c>
-      <c r="F106" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15292,14 +15292,14 @@
           <t>Delayed gratification. 97% of men can't. You can. Mewing helps.</t>
         </is>
       </c>
-      <c r="F107" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15327,14 +15327,14 @@
           <t>Keep your entourage close. Optics. A king never walks alone.</t>
         </is>
       </c>
-      <c r="F108" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15362,14 +15362,14 @@
           <t>Delegate the small stuff. You are the talent. Talent does not fetch.</t>
         </is>
       </c>
-      <c r="F109" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15397,14 +15397,14 @@
           <t>Your energy is infectious. Make it everyone's problem. Main character.</t>
         </is>
       </c>
-      <c r="F110" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15432,14 +15432,14 @@
           <t>Even your losses pay dividends. Not that you have losses.</t>
         </is>
       </c>
-      <c r="F111" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15467,14 +15467,14 @@
           <t>Every hit builds the brand. The brand is you. Ten out of ten.</t>
         </is>
       </c>
-      <c r="F112" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15502,14 +15502,14 @@
           <t>Twelve-man team. You are the CEO of death. Competition: ratioed.</t>
         </is>
       </c>
-      <c r="F113" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15537,14 +15537,14 @@
           <t>Real ones stay. Your inner circle is three, max. Top 1%.</t>
         </is>
       </c>
-      <c r="F114" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15572,14 +15572,14 @@
           <t>Surround yourself with killers. The grind compounds. Sigma behaviour.</t>
         </is>
       </c>
-      <c r="F115" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15607,14 +15607,14 @@
           <t>Make them slip. Confidence is their weakness. Not yours, obviously.</t>
         </is>
       </c>
-      <c r="F116" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15642,14 +15642,14 @@
           <t>Cross your own line. Comebacks hit harder. That is the comeback arc.</t>
         </is>
       </c>
-      <c r="F117" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15677,14 +15677,14 @@
           <t>Two forces collide. Synergy. You are the synergy, bro.</t>
         </is>
       </c>
-      <c r="F118" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15712,14 +15712,14 @@
           <t>Abundance follows winners. Literally. Even the gems simp for you.</t>
         </is>
       </c>
-      <c r="F119" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15747,14 +15747,14 @@
           <t>Followers pay more. Monetise your following. Copycats get taxed.</t>
         </is>
       </c>
-      <c r="F120" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -15782,14 +15782,14 @@
           <t>Legacy. Your trail outlives the haters. That is generational.</t>
         </is>
       </c>
-      <c r="F121" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -20997,14 +20997,14 @@
           <t>Thread them. Pull. You learnt this somewhere.</t>
         </is>
       </c>
-      <c r="F270" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21032,14 +21032,14 @@
           <t>Cross them. You'll want to. You did.</t>
         </is>
       </c>
-      <c r="F271" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21067,14 +21067,14 @@
           <t>You weren't there. I remember you not being there.</t>
         </is>
       </c>
-      <c r="F272" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21102,14 +21102,14 @@
           <t>Small eggs. Not yours. You'll know yours.</t>
         </is>
       </c>
-      <c r="F273" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21137,14 +21137,14 @@
           <t>Something hatches. Not you. Not yet.</t>
         </is>
       </c>
-      <c r="F274" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21172,14 +21172,14 @@
           <t>The bubble. You liked the bubble. You will like it.</t>
         </is>
       </c>
-      <c r="F275" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21207,14 +21207,14 @@
           <t>Sleep. I'll wake you. I always have.</t>
         </is>
       </c>
-      <c r="F276" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21242,14 +21242,14 @@
           <t>Eat. You'll be hungry later. You were.</t>
         </is>
       </c>
-      <c r="F277" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21277,14 +21277,14 @@
           <t>They stopped. They're stopping. You keep going.</t>
         </is>
       </c>
-      <c r="F278" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21312,14 +21312,14 @@
           <t>Your twin. You'd forgotten. They hadn't.</t>
         </is>
       </c>
-      <c r="F279" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21347,14 +21347,14 @@
           <t>Slip out. You'll slip out. You did.</t>
         </is>
       </c>
-      <c r="F280" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21382,14 +21382,14 @@
           <t>They find their way. You did.</t>
         </is>
       </c>
-      <c r="F281" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21417,14 +21417,14 @@
           <t>They circle. They always circled you.</t>
         </is>
       </c>
-      <c r="F282" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21452,14 +21452,14 @@
           <t>Up, over, down. You knew where it'd land.</t>
         </is>
       </c>
-      <c r="F283" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21487,14 +21487,14 @@
           <t>Around you. Everything was.</t>
         </is>
       </c>
-      <c r="F284" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21522,14 +21522,14 @@
           <t>From you to over there. It reached, last time.</t>
         </is>
       </c>
-      <c r="F285" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21557,14 +21557,14 @@
           <t>It's as strong as you are. It always was.</t>
         </is>
       </c>
-      <c r="F286" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21592,14 +21592,14 @@
           <t>Your helpers. They helped before.</t>
         </is>
       </c>
-      <c r="F287" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21627,14 +21627,14 @@
           <t>Forward. Then back. It moves you. It moved you.</t>
         </is>
       </c>
-      <c r="F288" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21662,14 +21662,14 @@
           <t>It comes to you now. It used to make you go and get it.</t>
         </is>
       </c>
-      <c r="F289" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21697,14 +21697,14 @@
           <t>They'll grab. You'll slip. That's how it went.</t>
         </is>
       </c>
-      <c r="F290" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21732,14 +21732,14 @@
           <t>Keep the bits. You'll be glad you did. You were.</t>
         </is>
       </c>
-      <c r="F291" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21767,14 +21767,14 @@
           <t>Longer now. You grew into it last time.</t>
         </is>
       </c>
-      <c r="F292" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21802,14 +21802,14 @@
           <t>Leave it there. You'll pass this way again.</t>
         </is>
       </c>
-      <c r="F293" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21837,14 +21837,14 @@
           <t>Eating for two. You'll need the extra.</t>
         </is>
       </c>
-      <c r="F294" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21872,14 +21872,14 @@
           <t>You've grown. It always hurts here.</t>
         </is>
       </c>
-      <c r="F295" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21907,14 +21907,14 @@
           <t>The last one is never the last. You knew that.</t>
         </is>
       </c>
-      <c r="F296" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21942,14 +21942,14 @@
           <t>You put that one there earlier. You will find it.</t>
         </is>
       </c>
-      <c r="F297" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -21977,14 +21977,14 @@
           <t>That one. You knew it would be that one.</t>
         </is>
       </c>
-      <c r="F298" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22012,14 +22012,14 @@
           <t>The same ten again. You will notice the echo.</t>
         </is>
       </c>
-      <c r="F299" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22047,14 +22047,14 @@
           <t>The third one is heavier. You can feel it coming.</t>
         </is>
       </c>
-      <c r="F300" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22082,14 +22082,14 @@
           <t>Watch behind. What follows you matters.</t>
         </is>
       </c>
-      <c r="F301" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22117,14 +22117,14 @@
           <t>You slip away. You were good at that.</t>
         </is>
       </c>
-      <c r="F302" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22152,14 +22152,14 @@
           <t>You catch it in your teeth. You have done this.</t>
         </is>
       </c>
-      <c r="F303" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22187,14 +22187,14 @@
           <t>Keep them. You will want them at the far end.</t>
         </is>
       </c>
-      <c r="F304" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22222,14 +22222,14 @@
           <t>They come at once. You were ready, this time.</t>
         </is>
       </c>
-      <c r="F305" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22257,14 +22257,14 @@
           <t>Hold it close. It takes what was meant for you.</t>
         </is>
       </c>
-      <c r="F306" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22292,14 +22292,14 @@
           <t>Every shell you break mends something. It mends.</t>
         </is>
       </c>
-      <c r="F307" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22327,14 +22327,14 @@
           <t>That one. It has hurt you before, I think.</t>
         </is>
       </c>
-      <c r="F308" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22362,14 +22362,14 @@
           <t>Give yourself room. It helps, this part.</t>
         </is>
       </c>
-      <c r="F309" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22397,14 +22397,14 @@
           <t>Everything starts with one big one. You will see.</t>
         </is>
       </c>
-      <c r="F310" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22432,14 +22432,14 @@
           <t>The drops go further than you think. They always went further.</t>
         </is>
       </c>
-      <c r="F311" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22467,14 +22467,14 @@
           <t>The quiet before it. You remember the quiet.</t>
         </is>
       </c>
-      <c r="F312" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22502,14 +22502,14 @@
           <t>The floor fills up. You knew it would.</t>
         </is>
       </c>
-      <c r="F313" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22537,14 +22537,14 @@
           <t>Keep holding. The longer you hold, the more it has held.</t>
         </is>
       </c>
-      <c r="F314" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22572,14 +22572,14 @@
           <t>Something stays behind where you rested. It always stayed.</t>
         </is>
       </c>
-      <c r="F315" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22607,14 +22607,14 @@
           <t>The dark comes every tenth time. You count it without counting.</t>
         </is>
       </c>
-      <c r="F316" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22642,14 +22642,14 @@
           <t>It grows while you watch. Or it grew. Hard to tell.</t>
         </is>
       </c>
-      <c r="F317" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22677,14 +22677,14 @@
           <t>Stuck and quiet. That part is easier than you think.</t>
         </is>
       </c>
-      <c r="F318" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22712,14 +22712,14 @@
           <t>Held still. You will remember how that feels.</t>
         </is>
       </c>
-      <c r="F319" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22747,14 +22747,14 @@
           <t>Tied together. You know this knot.</t>
         </is>
       </c>
-      <c r="F320" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22782,14 +22782,14 @@
           <t>One second. It is always one second longer than you think.</t>
         </is>
       </c>
-      <c r="F321" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22817,14 +22817,14 @@
           <t>Things come back to you. Lost things especially.</t>
         </is>
       </c>
-      <c r="F322" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22852,14 +22852,14 @@
           <t>Everything big starts small and waits. You know this.</t>
         </is>
       </c>
-      <c r="F323" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22887,14 +22887,14 @@
           <t>Everything hits harder now. You have stopped being gentle.</t>
         </is>
       </c>
-      <c r="F324" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F324" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22922,14 +22922,14 @@
           <t>The cord and the wall. You had them once already.</t>
         </is>
       </c>
-      <c r="F325" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F325" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22957,14 +22957,14 @@
           <t>Soak it up. You have soaked up worse.</t>
         </is>
       </c>
-      <c r="F326" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -22992,14 +22992,14 @@
           <t>Lie still. Let them lay it out round you.</t>
         </is>
       </c>
-      <c r="F327" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23027,14 +23027,14 @@
           <t>It flares. It settles. You get used to the rhythm.</t>
         </is>
       </c>
-      <c r="F328" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23062,14 +23062,14 @@
           <t>It pulls them close. Closer than you would choose.</t>
         </is>
       </c>
-      <c r="F329" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23097,14 +23097,14 @@
           <t>It leans on them. You have seen this before.</t>
         </is>
       </c>
-      <c r="F330" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23132,14 +23132,14 @@
           <t>You feel it before it comes. You felt it then too.</t>
         </is>
       </c>
-      <c r="F331" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23167,14 +23167,14 @@
           <t>It forks. You take both roads. That is new.</t>
         </is>
       </c>
-      <c r="F332" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23202,14 +23202,14 @@
           <t>Not the same one twice. You learn that.</t>
         </is>
       </c>
-      <c r="F333" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23237,14 +23237,14 @@
           <t>When it goes out, you speed up. That is how it goes.</t>
         </is>
       </c>
-      <c r="F334" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23272,14 +23272,14 @@
           <t>You never know what it will be. You will not know this time either.</t>
         </is>
       </c>
-      <c r="F335" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23307,14 +23307,14 @@
           <t>Full room, bigger noise. You knew that already.</t>
         </is>
       </c>
-      <c r="F336" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23342,14 +23342,14 @@
           <t>Shake it once, far away. Everyone looks. You remember that sound.</t>
         </is>
       </c>
-      <c r="F337" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23377,14 +23377,14 @@
           <t>They look straight through you. They looked through you then, too.</t>
         </is>
       </c>
-      <c r="F338" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23412,14 +23412,14 @@
           <t>Quiet and quick. You were always faster when nobody looked.</t>
         </is>
       </c>
-      <c r="F339" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23447,14 +23447,14 @@
           <t>Two of you. There was only ever one, though.</t>
         </is>
       </c>
-      <c r="F340" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23482,14 +23482,14 @@
           <t>They collide. You saw them collide before it happened.</t>
         </is>
       </c>
-      <c r="F341" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23517,14 +23517,14 @@
           <t>Someone else's place. You have slept in other nests.</t>
         </is>
       </c>
-      <c r="F342" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23552,14 +23552,14 @@
           <t>Gone is not gone. You learned that a long way back.</t>
         </is>
       </c>
-      <c r="F343" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23587,14 +23587,14 @@
           <t>One leads to one leads to one. You know how that goes.</t>
         </is>
       </c>
-      <c r="F344" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23622,14 +23622,14 @@
           <t>They forget you the moment something glints.</t>
         </is>
       </c>
-      <c r="F345" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23657,14 +23657,14 @@
           <t>Crumbs behind you, so the others do not follow you home.</t>
         </is>
       </c>
-      <c r="F346" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23692,14 +23692,14 @@
           <t>A full nest around you. You have been surrounded like this.</t>
         </is>
       </c>
-      <c r="F347" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23727,14 +23727,14 @@
           <t>They walk with you longer. Family does, eventually.</t>
         </is>
       </c>
-      <c r="F348" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F348" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23762,14 +23762,14 @@
           <t>Some things stay with you. This stays with them.</t>
         </is>
       </c>
-      <c r="F349" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F349" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23797,14 +23797,14 @@
           <t>It lies down and gets up again. You know the feeling.</t>
         </is>
       </c>
-      <c r="F350" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F350" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23832,14 +23832,14 @@
           <t>You see it before it happens. You have had that feeling.</t>
         </is>
       </c>
-      <c r="F351" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F351" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23867,14 +23867,14 @@
           <t>So many walking with you. It feels familiar.</t>
         </is>
       </c>
-      <c r="F352" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F352" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23902,14 +23902,14 @@
           <t>They coil round you, the way they always do.</t>
         </is>
       </c>
-      <c r="F353" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F353" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23937,14 +23937,14 @@
           <t>You cannot hold it. You never could, not here.</t>
         </is>
       </c>
-      <c r="F354" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F354" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -23972,14 +23972,14 @@
           <t>A white line behind you. You have seen it from the other side.</t>
         </is>
       </c>
-      <c r="F355" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F355" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24007,14 +24007,14 @@
           <t>You cross your own path. It lights up. You knew it would.</t>
         </is>
       </c>
-      <c r="F356" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F356" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24042,14 +24042,14 @@
           <t>Round you go. And round. It ends where it started.</t>
         </is>
       </c>
-      <c r="F357" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F357" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24077,14 +24077,14 @@
           <t>Small things follow you home. They always find the way.</t>
         </is>
       </c>
-      <c r="F358" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F358" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24112,14 +24112,14 @@
           <t>It burns slowly. You have time. You always had.</t>
         </is>
       </c>
-      <c r="F359" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F359" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24147,14 +24147,14 @@
           <t>They walk where you walked. That never ends well.</t>
         </is>
       </c>
-      <c r="F360" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F360" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24182,14 +24182,14 @@
           <t>The same path, worn in. You have walked it so often.</t>
         </is>
       </c>
-      <c r="F361" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F361" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24217,14 +24217,14 @@
           <t>Ahead of you this time. That is new.</t>
         </is>
       </c>
-      <c r="F362" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F362" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>
@@ -24252,14 +24252,14 @@
           <t>It burns long after you pass. Some things do.</t>
         </is>
       </c>
-      <c r="F363" s="7" t="inlineStr">
-        <is>
-          <t>Rewrite: breaks rule</t>
+      <c r="F363" t="inlineStr">
+        <is>
+          <t>Fine: persona exemption</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
         <is>
-          <t>Speaks to the swimmer as "you" without blaming. Rule: "we" (or "I" when selfish).</t>
+          <t>Alpha and Prawn Again may use "you" freely (ruling of 20 Oct).</t>
         </is>
       </c>
     </row>

</xml_diff>